<commit_message>
nu er databasen lavet i SQlquery filen i BD_projcet
</commit_message>
<xml_diff>
--- a/Budweg/BD_Projekt/Bakke.xlsx
+++ b/Budweg/BD_Projekt/Bakke.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MPH\Programmering\2.Semster\Budweg\BD_Projekt\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MPH\Programmering\2.Semster\Budweg_TeamB2\Budweg\BD_Projekt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF6E3E64-7A5C-4C2A-8D45-2CC23C0C3640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EBA39C0-DC9A-4904-A238-C57A3E890B3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="9420" xr2:uid="{D84736E9-C562-4EA0-9D8B-E53B397979CA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{D84736E9-C562-4EA0-9D8B-E53B397979CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,16 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="7">
-  <si>
-    <t>Bremse</t>
-  </si>
-  <si>
-    <t>EBPBremse</t>
-  </si>
-  <si>
-    <t>Reserve</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>BakkeID</t>
   </si>
@@ -57,6 +48,9 @@
   </si>
   <si>
     <t>WorkorderID</t>
+  </si>
+  <si>
+    <t>D</t>
   </si>
 </sst>
 </file>
@@ -469,87 +463,55 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1">
-        <v>30</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="1">
-        <v>1</v>
-      </c>
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" s="1">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="1">
         <v>1</v>
-      </c>
-      <c r="D3" s="1">
-        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1">
-        <v>7</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D4" s="1">
-        <v>4</v>
-      </c>
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
-        <v>4</v>
-      </c>
-      <c r="B5" s="1">
-        <v>11</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D5" s="1">
-        <v>5</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="1">
-        <v>5</v>
-      </c>
-      <c r="B6" s="1">
-        <v>13</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D6" s="1">
-        <v>2</v>
-      </c>
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>